<commit_message>
Refactorizacion y formateo del informe
</commit_message>
<xml_diff>
--- a/metrics.xlsx
+++ b/metrics.xlsx
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>7</v>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>99</v>
+        <v>131</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>21</v>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>128516</v>
+        <v>131968</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>103</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>110639</v>
+        <v>113422</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>434</v>
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>7427.272727272725</v>
+        <v>7427.272727272728</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>7256.374010775066</v>
+        <v>7238.948436030663</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>18175</v>
+        <v>21556</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>43</v>
@@ -769,13 +769,13 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>13199</v>
+        <v>18982</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>189</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16">
@@ -791,10 +791,10 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>5</v>
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>70</v>
+        <v>143</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>8</v>
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>331</v>
+        <v>413</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>8</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>228</v>
+        <v>341</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>24</v>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>10</v>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>315</v>
+        <v>367</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>30</v>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>6</v>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D35" s="8" t="n">
         <v>11</v>

</xml_diff>